<commit_message>
Eliminar metricas de tiempo separadas
</commit_message>
<xml_diff>
--- a/kp/tablas/tabla_descriptivos.xlsx
+++ b/kp/tablas/tabla_descriptivos.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:CS7"/>
+  <dimension ref="A1:CG7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -460,40 +460,30 @@
       </c>
       <c r="AX1" t="inlineStr">
         <is>
-          <t>t_cuantico</t>
+          <t>tiempo_por_eval</t>
         </is>
       </c>
       <c r="BD1" t="inlineStr">
         <is>
-          <t>t_clasico</t>
+          <t>total_evals</t>
         </is>
       </c>
       <c r="BJ1" t="inlineStr">
         <is>
-          <t>tiempo_por_eval</t>
+          <t>sqa_beta</t>
         </is>
       </c>
       <c r="BP1" t="inlineStr">
         <is>
-          <t>total_evals</t>
+          <t>sqa_gamma</t>
         </is>
       </c>
       <c r="BV1" t="inlineStr">
         <is>
-          <t>sqa_beta</t>
+          <t>sqa_trotter</t>
         </is>
       </c>
       <c r="CB1" t="inlineStr">
-        <is>
-          <t>sqa_gamma</t>
-        </is>
-      </c>
-      <c r="CH1" t="inlineStr">
-        <is>
-          <t>sqa_trotter</t>
-        </is>
-      </c>
-      <c r="CN1" t="inlineStr">
         <is>
           <t>sqa_num_sweeps</t>
         </is>
@@ -921,66 +911,6 @@
           <t>max</t>
         </is>
       </c>
-      <c r="CH2" t="inlineStr">
-        <is>
-          <t>count</t>
-        </is>
-      </c>
-      <c r="CI2" t="inlineStr">
-        <is>
-          <t>mean</t>
-        </is>
-      </c>
-      <c r="CJ2" t="inlineStr">
-        <is>
-          <t>median</t>
-        </is>
-      </c>
-      <c r="CK2" t="inlineStr">
-        <is>
-          <t>std</t>
-        </is>
-      </c>
-      <c r="CL2" t="inlineStr">
-        <is>
-          <t>min</t>
-        </is>
-      </c>
-      <c r="CM2" t="inlineStr">
-        <is>
-          <t>max</t>
-        </is>
-      </c>
-      <c r="CN2" t="inlineStr">
-        <is>
-          <t>count</t>
-        </is>
-      </c>
-      <c r="CO2" t="inlineStr">
-        <is>
-          <t>mean</t>
-        </is>
-      </c>
-      <c r="CP2" t="inlineStr">
-        <is>
-          <t>median</t>
-        </is>
-      </c>
-      <c r="CQ2" t="inlineStr">
-        <is>
-          <t>std</t>
-        </is>
-      </c>
-      <c r="CR2" t="inlineStr">
-        <is>
-          <t>min</t>
-        </is>
-      </c>
-      <c r="CS2" t="inlineStr">
-        <is>
-          <t>max</t>
-        </is>
-      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -996,7 +926,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="C4" t="n">
         <v>1</v>
@@ -1014,34 +944,34 @@
         <v>1</v>
       </c>
       <c r="H4" t="n">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="I4" t="n">
-        <v>5630.720799563635</v>
+        <v>6118.944805116252</v>
       </c>
       <c r="J4" t="n">
-        <v>1046.426593100012</v>
+        <v>1660.014493150025</v>
       </c>
       <c r="K4" t="n">
-        <v>6878.798538315412</v>
+        <v>7191.64290381582</v>
       </c>
       <c r="L4" t="n">
         <v>427.3249366999953</v>
       </c>
       <c r="M4" t="n">
-        <v>18664.43478180002</v>
+        <v>18865.49624790018</v>
       </c>
       <c r="N4" t="n">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="O4" t="n">
-        <v>0.7103896103896105</v>
+        <v>0.6975</v>
       </c>
       <c r="P4" t="n">
-        <v>0.8</v>
+        <v>0.75</v>
       </c>
       <c r="Q4" t="n">
-        <v>0.2337252185481329</v>
+        <v>0.2407661820737699</v>
       </c>
       <c r="R4" t="n">
         <v>0.2</v>
@@ -1058,7 +988,7 @@
       <c r="X4" t="inlineStr"/>
       <c r="Y4" t="inlineStr"/>
       <c r="Z4" t="n">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="AA4" t="n">
         <v>1</v>
@@ -1076,16 +1006,16 @@
         <v>1</v>
       </c>
       <c r="AF4" t="n">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="AG4" t="n">
-        <v>0.9462072380115858</v>
+        <v>0.9443768015297908</v>
       </c>
       <c r="AH4" t="n">
-        <v>0.9555555555555556</v>
+        <v>0.9463095238095238</v>
       </c>
       <c r="AI4" t="n">
-        <v>0.04370264339242058</v>
+        <v>0.04405147770415568</v>
       </c>
       <c r="AJ4" t="n">
         <v>0.8</v>
@@ -1094,7 +1024,7 @@
         <v>1</v>
       </c>
       <c r="AL4" t="n">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="AM4" t="n">
         <v>10</v>
@@ -1120,77 +1050,57 @@
       <c r="AV4" t="inlineStr"/>
       <c r="AW4" t="inlineStr"/>
       <c r="AX4" t="n">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="AY4" t="n">
-        <v>5617.777592793516</v>
+        <v>2.437825256508965</v>
       </c>
       <c r="AZ4" t="n">
-        <v>1036.494622999278</v>
+        <v>0.6613590577091795</v>
       </c>
       <c r="BA4" t="n">
-        <v>6874.614064101911</v>
+        <v>2.865196199266355</v>
       </c>
       <c r="BB4" t="n">
-        <v>418.1754300994217</v>
+        <v>0.1702478349402238</v>
       </c>
       <c r="BC4" t="n">
-        <v>18643.63132550102</v>
+        <v>7.516132199362596</v>
       </c>
       <c r="BD4" t="n">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="BE4" t="n">
-        <v>12.94060618699794</v>
+        <v>2510</v>
       </c>
       <c r="BF4" t="n">
-        <v>10.07857049943414</v>
+        <v>2510</v>
       </c>
       <c r="BG4" t="n">
-        <v>4.254139947572392</v>
+        <v>0</v>
       </c>
       <c r="BH4" t="n">
-        <v>8.885841900017112</v>
+        <v>2510</v>
       </c>
       <c r="BI4" t="n">
-        <v>20.81608179747127</v>
+        <v>2510</v>
       </c>
       <c r="BJ4" t="n">
-        <v>77</v>
-      </c>
-      <c r="BK4" t="n">
-        <v>2.243313714934029</v>
-      </c>
-      <c r="BL4" t="n">
-        <v>0.4169017183266958</v>
-      </c>
-      <c r="BM4" t="n">
-        <v>2.740557022115692</v>
-      </c>
-      <c r="BN4" t="n">
-        <v>0.1702478349402238</v>
-      </c>
-      <c r="BO4" t="n">
-        <v>7.43602811294836</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="BK4" t="inlineStr"/>
+      <c r="BL4" t="inlineStr"/>
+      <c r="BM4" t="inlineStr"/>
+      <c r="BN4" t="inlineStr"/>
+      <c r="BO4" t="inlineStr"/>
       <c r="BP4" t="n">
-        <v>77</v>
-      </c>
-      <c r="BQ4" t="n">
-        <v>2510</v>
-      </c>
-      <c r="BR4" t="n">
-        <v>2510</v>
-      </c>
-      <c r="BS4" t="n">
-        <v>0</v>
-      </c>
-      <c r="BT4" t="n">
-        <v>2510</v>
-      </c>
-      <c r="BU4" t="n">
-        <v>2510</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="BQ4" t="inlineStr"/>
+      <c r="BR4" t="inlineStr"/>
+      <c r="BS4" t="inlineStr"/>
+      <c r="BT4" t="inlineStr"/>
+      <c r="BU4" t="inlineStr"/>
       <c r="BV4" t="n">
         <v>0</v>
       </c>
@@ -1207,22 +1117,6 @@
       <c r="CE4" t="inlineStr"/>
       <c r="CF4" t="inlineStr"/>
       <c r="CG4" t="inlineStr"/>
-      <c r="CH4" t="n">
-        <v>0</v>
-      </c>
-      <c r="CI4" t="inlineStr"/>
-      <c r="CJ4" t="inlineStr"/>
-      <c r="CK4" t="inlineStr"/>
-      <c r="CL4" t="inlineStr"/>
-      <c r="CM4" t="inlineStr"/>
-      <c r="CN4" t="n">
-        <v>0</v>
-      </c>
-      <c r="CO4" t="inlineStr"/>
-      <c r="CP4" t="inlineStr"/>
-      <c r="CQ4" t="inlineStr"/>
-      <c r="CR4" t="inlineStr"/>
-      <c r="CS4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1358,74 +1252,54 @@
         <v>80</v>
       </c>
       <c r="AY5" t="n">
-        <v>3723.54779203602</v>
+        <v>1.48853499528784</v>
       </c>
       <c r="AZ5" t="n">
-        <v>1427.980824149476</v>
+        <v>0.5731432319123648</v>
       </c>
       <c r="BA5" t="n">
-        <v>3782.479975892104</v>
+        <v>1.508468351271774</v>
       </c>
       <c r="BB5" t="n">
-        <v>367.9535155003541</v>
+        <v>0.1502419291234591</v>
       </c>
       <c r="BC5" t="n">
-        <v>10430.45848029782</v>
+        <v>4.16319847386451</v>
       </c>
       <c r="BD5" t="n">
         <v>80</v>
       </c>
       <c r="BE5" t="n">
-        <v>12.67577020770841</v>
+        <v>2510</v>
       </c>
       <c r="BF5" t="n">
-        <v>10.39796809953987</v>
+        <v>2510</v>
       </c>
       <c r="BG5" t="n">
-        <v>3.786864914705294</v>
+        <v>0</v>
       </c>
       <c r="BH5" t="n">
-        <v>9.058024600963108</v>
+        <v>2510</v>
       </c>
       <c r="BI5" t="n">
-        <v>19.80072690383531</v>
+        <v>2510</v>
       </c>
       <c r="BJ5" t="n">
-        <v>80</v>
-      </c>
-      <c r="BK5" t="n">
-        <v>1.48853499528784</v>
-      </c>
-      <c r="BL5" t="n">
-        <v>0.5731432319123648</v>
-      </c>
-      <c r="BM5" t="n">
-        <v>1.508468351271774</v>
-      </c>
-      <c r="BN5" t="n">
-        <v>0.1502419291234591</v>
-      </c>
-      <c r="BO5" t="n">
-        <v>4.16319847386451</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="BK5" t="inlineStr"/>
+      <c r="BL5" t="inlineStr"/>
+      <c r="BM5" t="inlineStr"/>
+      <c r="BN5" t="inlineStr"/>
+      <c r="BO5" t="inlineStr"/>
       <c r="BP5" t="n">
-        <v>80</v>
-      </c>
-      <c r="BQ5" t="n">
-        <v>2510</v>
-      </c>
-      <c r="BR5" t="n">
-        <v>2510</v>
-      </c>
-      <c r="BS5" t="n">
-        <v>0</v>
-      </c>
-      <c r="BT5" t="n">
-        <v>2510</v>
-      </c>
-      <c r="BU5" t="n">
-        <v>2510</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="BQ5" t="inlineStr"/>
+      <c r="BR5" t="inlineStr"/>
+      <c r="BS5" t="inlineStr"/>
+      <c r="BT5" t="inlineStr"/>
+      <c r="BU5" t="inlineStr"/>
       <c r="BV5" t="n">
         <v>0</v>
       </c>
@@ -1442,22 +1316,6 @@
       <c r="CE5" t="inlineStr"/>
       <c r="CF5" t="inlineStr"/>
       <c r="CG5" t="inlineStr"/>
-      <c r="CH5" t="n">
-        <v>0</v>
-      </c>
-      <c r="CI5" t="inlineStr"/>
-      <c r="CJ5" t="inlineStr"/>
-      <c r="CK5" t="inlineStr"/>
-      <c r="CL5" t="inlineStr"/>
-      <c r="CM5" t="inlineStr"/>
-      <c r="CN5" t="n">
-        <v>0</v>
-      </c>
-      <c r="CO5" t="inlineStr"/>
-      <c r="CP5" t="inlineStr"/>
-      <c r="CQ5" t="inlineStr"/>
-      <c r="CR5" t="inlineStr"/>
-      <c r="CS5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1466,7 +1324,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="C6" t="n">
         <v>1</v>
@@ -1484,16 +1342,16 @@
         <v>1</v>
       </c>
       <c r="H6" t="n">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="I6" t="n">
-        <v>0.02103277630981444</v>
+        <v>0.02132685249380296</v>
       </c>
       <c r="J6" t="n">
-        <v>0.0204065999714657</v>
+        <v>0.02071459998842325</v>
       </c>
       <c r="K6" t="n">
-        <v>0.003916212504046863</v>
+        <v>0.004033049681927782</v>
       </c>
       <c r="L6" t="n">
         <v>0.0155887999571859</v>
@@ -1502,16 +1360,16 @@
         <v>0.0307911001145839</v>
       </c>
       <c r="N6" t="n">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="O6" t="n">
-        <v>0.8118421052631579</v>
+        <v>0.8025</v>
       </c>
       <c r="P6" t="n">
         <v>0.9</v>
       </c>
       <c r="Q6" t="n">
-        <v>0.219676796081976</v>
+        <v>0.2198820166949147</v>
       </c>
       <c r="R6" t="n">
         <v>0.3</v>
@@ -1520,16 +1378,16 @@
         <v>1</v>
       </c>
       <c r="T6" t="n">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="U6" t="n">
-        <v>0.2331578947368421</v>
+        <v>0.22575</v>
       </c>
       <c r="V6" t="n">
-        <v>0.23</v>
+        <v>0.225</v>
       </c>
       <c r="W6" t="n">
-        <v>0.1487567188516498</v>
+        <v>0.148960745827444</v>
       </c>
       <c r="X6" t="n">
         <v>0.03</v>
@@ -1538,16 +1396,16 @@
         <v>0.5600000000000001</v>
       </c>
       <c r="Z6" t="n">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="AA6" t="n">
-        <v>0.9899999999999999</v>
+        <v>0.9898749999999999</v>
       </c>
       <c r="AB6" t="n">
         <v>1</v>
       </c>
       <c r="AC6" t="n">
-        <v>0.01336662510384228</v>
+        <v>0.01354726839671593</v>
       </c>
       <c r="AD6" t="n">
         <v>0.9399999999999999</v>
@@ -1556,16 +1414,16 @@
         <v>1</v>
       </c>
       <c r="AF6" t="n">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="AG6" t="n">
-        <v>0.6212515525767222</v>
+        <v>0.6228070581958244</v>
       </c>
       <c r="AH6" t="n">
-        <v>0.615880808080808</v>
+        <v>0.6194909090909091</v>
       </c>
       <c r="AI6" t="n">
-        <v>0.06936106495930626</v>
+        <v>0.06826337927483085</v>
       </c>
       <c r="AJ6" t="n">
         <v>0.43625</v>
@@ -1574,7 +1432,7 @@
         <v>0.7557142857142857</v>
       </c>
       <c r="AL6" t="n">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="AM6" t="n">
         <v>10</v>
@@ -1592,7 +1450,7 @@
         <v>10</v>
       </c>
       <c r="AR6" t="n">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="AS6" t="n">
         <v>100</v>
@@ -1657,22 +1515,6 @@
       <c r="CE6" t="inlineStr"/>
       <c r="CF6" t="inlineStr"/>
       <c r="CG6" t="inlineStr"/>
-      <c r="CH6" t="n">
-        <v>0</v>
-      </c>
-      <c r="CI6" t="inlineStr"/>
-      <c r="CJ6" t="inlineStr"/>
-      <c r="CK6" t="inlineStr"/>
-      <c r="CL6" t="inlineStr"/>
-      <c r="CM6" t="inlineStr"/>
-      <c r="CN6" t="n">
-        <v>0</v>
-      </c>
-      <c r="CO6" t="inlineStr"/>
-      <c r="CP6" t="inlineStr"/>
-      <c r="CQ6" t="inlineStr"/>
-      <c r="CR6" t="inlineStr"/>
-      <c r="CS6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1841,21 +1683,41 @@
       <c r="BH7" t="inlineStr"/>
       <c r="BI7" t="inlineStr"/>
       <c r="BJ7" t="n">
-        <v>0</v>
-      </c>
-      <c r="BK7" t="inlineStr"/>
-      <c r="BL7" t="inlineStr"/>
-      <c r="BM7" t="inlineStr"/>
-      <c r="BN7" t="inlineStr"/>
-      <c r="BO7" t="inlineStr"/>
+        <v>80</v>
+      </c>
+      <c r="BK7" t="n">
+        <v>10</v>
+      </c>
+      <c r="BL7" t="n">
+        <v>10</v>
+      </c>
+      <c r="BM7" t="n">
+        <v>0</v>
+      </c>
+      <c r="BN7" t="n">
+        <v>10</v>
+      </c>
+      <c r="BO7" t="n">
+        <v>10</v>
+      </c>
       <c r="BP7" t="n">
-        <v>0</v>
-      </c>
-      <c r="BQ7" t="inlineStr"/>
-      <c r="BR7" t="inlineStr"/>
-      <c r="BS7" t="inlineStr"/>
-      <c r="BT7" t="inlineStr"/>
-      <c r="BU7" t="inlineStr"/>
+        <v>80</v>
+      </c>
+      <c r="BQ7" t="n">
+        <v>1</v>
+      </c>
+      <c r="BR7" t="n">
+        <v>1</v>
+      </c>
+      <c r="BS7" t="n">
+        <v>0</v>
+      </c>
+      <c r="BT7" t="n">
+        <v>1</v>
+      </c>
+      <c r="BU7" t="n">
+        <v>1</v>
+      </c>
       <c r="BV7" t="n">
         <v>80</v>
       </c>
@@ -1878,59 +1740,23 @@
         <v>80</v>
       </c>
       <c r="CC7" t="n">
-        <v>1</v>
+        <v>1000</v>
       </c>
       <c r="CD7" t="n">
-        <v>1</v>
+        <v>1000</v>
       </c>
       <c r="CE7" t="n">
         <v>0</v>
       </c>
       <c r="CF7" t="n">
-        <v>1</v>
+        <v>1000</v>
       </c>
       <c r="CG7" t="n">
-        <v>1</v>
-      </c>
-      <c r="CH7" t="n">
-        <v>80</v>
-      </c>
-      <c r="CI7" t="n">
-        <v>10</v>
-      </c>
-      <c r="CJ7" t="n">
-        <v>10</v>
-      </c>
-      <c r="CK7" t="n">
-        <v>0</v>
-      </c>
-      <c r="CL7" t="n">
-        <v>10</v>
-      </c>
-      <c r="CM7" t="n">
-        <v>10</v>
-      </c>
-      <c r="CN7" t="n">
-        <v>80</v>
-      </c>
-      <c r="CO7" t="n">
-        <v>1000</v>
-      </c>
-      <c r="CP7" t="n">
-        <v>1000</v>
-      </c>
-      <c r="CQ7" t="n">
-        <v>0</v>
-      </c>
-      <c r="CR7" t="n">
-        <v>1000</v>
-      </c>
-      <c r="CS7" t="n">
         <v>1000</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="16">
+  <mergeCells count="14">
     <mergeCell ref="Z1:AE1"/>
     <mergeCell ref="H1:M1"/>
     <mergeCell ref="AF1:AK1"/>
@@ -1941,11 +1767,9 @@
     <mergeCell ref="BJ1:BO1"/>
     <mergeCell ref="CB1:CG1"/>
     <mergeCell ref="AL1:AQ1"/>
-    <mergeCell ref="CH1:CM1"/>
     <mergeCell ref="B1:G1"/>
     <mergeCell ref="BP1:BU1"/>
     <mergeCell ref="BV1:CA1"/>
-    <mergeCell ref="CN1:CS1"/>
     <mergeCell ref="N1:S1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>